<commit_message>
docs(MAPA-ORG-001): D3 — Jonathan Barbosa como auditor de GQA de projeto (v1.5)
Resolve a NC da auditoria "auditor de GQA do projeto nao consta na matriz org".
- §5 (GQA / Qualidade do Processo): Equipe passa a incluir Jonathan Barbosa
  (auditor de GQA de projeto — AASP_AndamentosProcessuais e AASP_CNJ); Flavio
  Fernandes mantido como titular organizacional (modelo de 2 niveis).
- Evidencia: auditorias de projeto em GQA-AASPAP01-001 e GQA-AASPCNJ01-001.
- .md, .docx e .xlsx atualizados; versao 1.4 -> 1.5 + linha de revisao.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mps-nivel-c/oficial/05_capacidade/MAPA-ORG-001_Matriz-de-Papeis-e-Responsabilidades.xlsx
+++ b/mps-nivel-c/oficial/05_capacidade/MAPA-ORG-001_Matriz-de-Papeis-e-Responsabilidades.xlsx
@@ -481,6 +481,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -796,6 +797,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1063,6 +1065,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -1190,12 +1193,12 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Flávio Fernandes</t>
+          <t>Flávio Fernandes (titular org); Jonathan Barbosa (auditor de GQA de projeto)</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>CV (Azure Architect Expert, TOGAF, COBIT, MBA FGV); REG-CAP-007/009</t>
+          <t>CV Flávio (Azure Architect Expert, TOGAF, COBIT, MBA FGV); REG-CAP-007/009; auditorias de projeto em GQA-AASPAP01-001 e GQA-AASPCNJ01-001 (Jonathan Barbosa)</t>
         </is>
       </c>
     </row>

</xml_diff>